<commit_message>
Migrate JSW Group homepage to Edge Delivery blocks
Replace the initial Maruti Suzuki scaffolding with the JSW Group homepage
migration: hero, group-overview stats, business-divisions carousel,
sustainability band, latest news, foundation (text + focus carousel),
full-width sports video, and careers teaser. Includes matching importer
parsers/transformers, page template, and brand tokens.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["carousel-banner","cards-channel","cards-highlight","carousel-product","carousel-product","cards-values","cards-counter"]</t>
+    <t>["carousel-hero","cards-stats","carousel-business","cards-news","foundation","video-bg","sustainability","disclaimer-modal"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,13 +52,13 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-05-14T11:36:34.762Z</t>
-  </si>
-  <si>
-    <t>Maruti Suzuki India Corporate - Discover Arena, NEXA cars, Commercial and True Value</t>
-  </si>
-  <si>
-    <t>https://www.marutisuzuki.com/</t>
+    <t>2026-07-20T11:20:14.782Z</t>
+  </si>
+  <si>
+    <t>JSW Group | Transforming Steel, Energy &amp; Cement Industries</t>
+  </si>
+  <si>
+    <t>https://www.jsw.in/</t>
   </si>
 </sst>
 </file>
@@ -456,7 +456,7 @@
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="31" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>